<commit_message>
feat: update GBT competency terminology, counter, and Excel template
</commit_message>
<xml_diff>
--- a/elearning-webapp/public/templates/gbt_competency_template.xlsx
+++ b/elearning-webapp/public/templates/gbt_competency_template.xlsx
@@ -404,7 +404,7 @@
         <v>กลุ่มระดับ GBT (levelGroup)</v>
       </c>
       <c r="B1" t="str">
-        <v>ชนิดสมรรถนะ (competencyType)</v>
+        <v>ประเภท (Competency Type) (ความรู้/ทักษะ/สมรรถนะ)</v>
       </c>
       <c r="C1" t="str">
         <v>ชื่อหมวดหมู่ย่อย (categoryName)</v>
@@ -413,7 +413,7 @@
         <v>รหัสสมรรถนะหลัก (code)</v>
       </c>
       <c r="E1" t="str">
-        <v>บทบาทงาน (sourceRole)</v>
+        <v>แหล่งที่มา / Role</v>
       </c>
       <c r="F1" t="str">
         <v>รหัสสมรรถนะเดิม (legacyCode)</v>

</xml_diff>